<commit_message>
Note live-formula behaviour on the scope summary tab
The summary counts are formulas with no cached values, so previewers
that only read cached values render them blank. Adds a line saying they
compute on open, and tidies a truncated column header.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019QqpDyTEkQXkQyKwAEgCh7
</commit_message>
<xml_diff>
--- a/gtm/work-copilot-feature-inventory.xlsx
+++ b/gtm/work-copilot-feature-inventory.xlsx
@@ -188,6 +188,9 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -214,9 +217,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8471,6 +8471,13 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>These cells are live formulas. They compute the moment the file opens in Excel, LibreOffice, Numbers or Google Sheets - if a preview shows them blank, that preview is not calculating, not a broken sheet.</t>
+        </is>
+      </c>
+    </row>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -8479,29 +8486,29 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C6" s="21" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="D6" s="21" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>Yours</t>
         </is>
       </c>
-      <c r="E6" s="21" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>What it means for the launch</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>Keep - core</t>
         </is>
@@ -8521,7 +8528,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>Keep - flag off by default</t>
         </is>
@@ -8541,7 +8548,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>Fix before launch</t>
         </is>
@@ -8561,7 +8568,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="25" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Extract to add-on</t>
         </is>
@@ -8581,7 +8588,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>Move to backup repo</t>
         </is>
@@ -8601,7 +8608,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="27" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>Delete</t>
         </is>
@@ -8621,20 +8628,20 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="29" t="inlineStr">
         <is>
           <t>Total features catalogued</t>
         </is>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="29">
         <f>COUNTA('Feature inventory'!$D$2:$D$130)</f>
         <v/>
       </c>
-      <c r="D13" s="28">
+      <c r="D13" s="29">
         <f>COUNTA('Feature inventory'!$L$2:$L$130)</f>
         <v/>
       </c>
-      <c r="E13" s="29" t="inlineStr">
+      <c r="E13" s="30" t="inlineStr">
         <is>
           <t>Column D of the inventory; 'Yours' counts decisions made so far.</t>
         </is>
@@ -8648,24 +8655,24 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <t>Bundle</t>
         </is>
       </c>
-      <c r="C17" s="21" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>Features</t>
         </is>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
         <is>
           <t>Keep - core</t>
         </is>
       </c>
-      <c r="E17" s="21" t="inlineStr">
-        <is>
-          <t>Share of the catalogue that is proposed core</t>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>Share proposed as core</t>
         </is>
       </c>
     </row>
@@ -8683,7 +8690,7 @@
         <f>COUNTIFS('Feature inventory'!$B$2:$B$130,$B18,'Feature inventory'!$J$2:$J$130,"Keep - core")</f>
         <v/>
       </c>
-      <c r="E18" s="30">
+      <c r="E18" s="31">
         <f>IF($C18=0,0,$D18/$C18)</f>
         <v/>
       </c>
@@ -8702,7 +8709,7 @@
         <f>COUNTIFS('Feature inventory'!$B$2:$B$130,$B19,'Feature inventory'!$J$2:$J$130,"Keep - core")</f>
         <v/>
       </c>
-      <c r="E19" s="30">
+      <c r="E19" s="31">
         <f>IF($C19=0,0,$D19/$C19)</f>
         <v/>
       </c>
@@ -8721,7 +8728,7 @@
         <f>COUNTIFS('Feature inventory'!$B$2:$B$130,$B20,'Feature inventory'!$J$2:$J$130,"Keep - core")</f>
         <v/>
       </c>
-      <c r="E20" s="30">
+      <c r="E20" s="31">
         <f>IF($C20=0,0,$D20/$C20)</f>
         <v/>
       </c>
@@ -8740,7 +8747,7 @@
         <f>COUNTIFS('Feature inventory'!$B$2:$B$130,$B21,'Feature inventory'!$J$2:$J$130,"Keep - core")</f>
         <v/>
       </c>
-      <c r="E21" s="30">
+      <c r="E21" s="31">
         <f>IF($C21=0,0,$D21/$C21)</f>
         <v/>
       </c>
@@ -8759,7 +8766,7 @@
         <f>COUNTIFS('Feature inventory'!$B$2:$B$130,$B22,'Feature inventory'!$J$2:$J$130,"Keep - core")</f>
         <v/>
       </c>
-      <c r="E22" s="30">
+      <c r="E22" s="31">
         <f>IF($C22=0,0,$D22/$C22)</f>
         <v/>
       </c>
@@ -8778,7 +8785,7 @@
         <f>COUNTIFS('Feature inventory'!$B$2:$B$130,$B23,'Feature inventory'!$J$2:$J$130,"Keep - core")</f>
         <v/>
       </c>
-      <c r="E23" s="30">
+      <c r="E23" s="31">
         <f>IF($C23=0,0,$D23/$C23)</f>
         <v/>
       </c>
@@ -8797,7 +8804,7 @@
         <f>COUNTIFS('Feature inventory'!$B$2:$B$130,$B24,'Feature inventory'!$J$2:$J$130,"Keep - core")</f>
         <v/>
       </c>
-      <c r="E24" s="30">
+      <c r="E24" s="31">
         <f>IF($C24=0,0,$D24/$C24)</f>
         <v/>
       </c>
@@ -8816,7 +8823,7 @@
         <f>COUNTIFS('Feature inventory'!$B$2:$B$130,$B25,'Feature inventory'!$J$2:$J$130,"Keep - core")</f>
         <v/>
       </c>
-      <c r="E25" s="30">
+      <c r="E25" s="31">
         <f>IF($C25=0,0,$D25/$C25)</f>
         <v/>
       </c>
@@ -8850,10 +8857,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B29:E29"/>
     <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B4:E4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8891,27 +8899,27 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>Blocker</t>
         </is>
       </c>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>Why it blocks</t>
         </is>
       </c>
-      <c r="E5" s="21" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="F5" s="21" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>Your owner</t>
         </is>
@@ -8931,7 +8939,7 @@
           <t>Core workspace UI lives in the theme. WP.org distributes plugins and themes separately, so 'install the plugin' does not currently give anyone a working product. Decide: bundle the UI into the plugin, or ship an explicit plugin+theme pair.</t>
         </is>
       </c>
-      <c r="E6" s="27" t="inlineStr">
+      <c r="E6" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -8952,7 +8960,7 @@
           <t>Personal server infrastructure in shippable code. Immediate rejection, and an embarrassment in a public repo.</t>
         </is>
       </c>
-      <c r="E7" s="27" t="inlineStr">
+      <c r="E7" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -8973,7 +8981,7 @@
           <t>Public repo would expose the author's server address.</t>
         </is>
       </c>
-      <c r="E8" s="27" t="inlineStr">
+      <c r="E8" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -8994,7 +9002,7 @@
           <t>Directly-accessible PHP outside the WordPress bootstrap. WP.org rejects this pattern.</t>
         </is>
       </c>
-      <c r="E9" s="27" t="inlineStr">
+      <c r="E9" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -9015,7 +9023,7 @@
           <t>Author's own tweet and bookmark CSVs, plus editor lock files, committed to the repo.</t>
         </is>
       </c>
-      <c r="E10" s="27" t="inlineStr">
+      <c r="E10" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -9036,7 +9044,7 @@
           <t>At least one endpoint uses __return_true. Every one of ~50 endpoints needs an explicit capability check.</t>
         </is>
       </c>
-      <c r="E11" s="27" t="inlineStr">
+      <c r="E11" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -9057,7 +9065,7 @@
           <t>WP.org forbids enqueuing assets from third-party CDNs. Also leaks every visitor's IP to a third party. Bundle both locally with their licence files.</t>
         </is>
       </c>
-      <c r="E12" s="27" t="inlineStr">
+      <c r="E12" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -9078,7 +9086,7 @@
           <t>wcp_db_version is stored but never compared on update, so a plugin upgrade never migrates an existing install's schema. This breaks people silently, and only after they have data worth losing.</t>
         </is>
       </c>
-      <c r="E13" s="24" t="inlineStr">
+      <c r="E13" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -9099,7 +9107,7 @@
           <t>Five custom tables are created with no cleanup path and no schema version guard. Reviewers check for this.</t>
         </is>
       </c>
-      <c r="E14" s="24" t="inlineStr">
+      <c r="E14" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -9120,7 +9128,7 @@
           <t>A theme silently changing site-wide REST behaviour will break other plugins. Move to the plugin, scope to this namespace.</t>
         </is>
       </c>
-      <c r="E15" s="24" t="inlineStr">
+      <c r="E15" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -9141,7 +9149,7 @@
           <t>Table grows unbounded and stores full prompts. It is named in readme.txt as a privacy feature, so it has to hold up.</t>
         </is>
       </c>
-      <c r="E16" s="24" t="inlineStr">
+      <c r="E16" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -9162,7 +9170,7 @@
           <t>Already patched twice (see changelog). Highest blast radius of any AI action - it rewrites many items at once.</t>
         </is>
       </c>
-      <c r="E17" s="24" t="inlineStr">
+      <c r="E17" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -9183,7 +9191,7 @@
           <t>AI-produced markdown rendered to the page. Confirm escaping before anyone else runs this.</t>
         </is>
       </c>
-      <c r="E18" s="24" t="inlineStr">
+      <c r="E18" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -9204,7 +9212,7 @@
           <t>Destructive and irreversible from the UI. Snapshot to a WP revision first.</t>
         </is>
       </c>
-      <c r="E19" s="24" t="inlineStr">
+      <c r="E19" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -9225,7 +9233,7 @@
           <t>No retry, no backoff, thin error surfacing. BYO-key is the headline USP - a bad key must produce a clear message, not a silent failure.</t>
         </is>
       </c>
-      <c r="E20" s="24" t="inlineStr">
+      <c r="E20" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -9246,7 +9254,7 @@
           <t>Model list will rot with each release. Move to a filterable config array.</t>
         </is>
       </c>
-      <c r="E21" s="23" t="inlineStr">
+      <c r="E21" s="24" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -9267,7 +9275,7 @@
           <t>Save latency and API cost on every edit. Queue it.</t>
         </is>
       </c>
-      <c r="E22" s="23" t="inlineStr">
+      <c r="E22" s="24" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -9288,7 +9296,7 @@
           <t>'Entire corpus' quietly does nothing. Must explain itself in the UI.</t>
         </is>
       </c>
-      <c r="E23" s="23" t="inlineStr">
+      <c r="E23" s="24" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -9309,7 +9317,7 @@
           <t>A headline USP is hidden in the admin area, contradicting the 'it all happens in a website' pitch.</t>
         </is>
       </c>
-      <c r="E24" s="23" t="inlineStr">
+      <c r="E24" s="24" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -9330,7 +9338,7 @@
           <t>The single biggest first-run comprehension risk in the product. Needs progressive disclosure.</t>
         </is>
       </c>
-      <c r="E25" s="23" t="inlineStr">
+      <c r="E25" s="24" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -9351,7 +9359,7 @@
           <t>Unusual interaction, likely broken on tablets. Verify or gate to pointer devices.</t>
         </is>
       </c>
-      <c r="E26" s="23" t="inlineStr">
+      <c r="E26" s="24" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -9372,7 +9380,7 @@
           <t>Author, contributor and URI fields still say 'Your Name' / 'yoursite.com'.</t>
         </is>
       </c>
-      <c r="E27" s="23" t="inlineStr">
+      <c r="E27" s="24" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -9393,7 +9401,7 @@
           <t>A redesign was committed then reverted. Marketing screenshots come from here - budget explicit design time.</t>
         </is>
       </c>
-      <c r="E28" s="23" t="inlineStr">
+      <c r="E28" s="24" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -9401,7 +9409,7 @@
       <c r="F28" s="15" t="n"/>
     </row>
     <row r="30">
-      <c r="C30" s="31" t="inlineStr">
+      <c r="C30" s="21" t="inlineStr">
         <is>
           <t>Severity key: Critical = cannot publish the repo or submit to WP.org. High = will produce data loss, a security report, or a bad first review. Medium = will cost adoption but is survivable.</t>
         </is>

</xml_diff>